<commit_message>
Actualizar datos Power Apps
</commit_message>
<xml_diff>
--- a/PowerApp_Data.xlsx
+++ b/PowerApp_Data.xlsx
@@ -673,12 +673,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -760,7 +760,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -1679,7 +1684,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -2011,12 +2021,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2435,12 +2440,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
+          <t>ARIZAPANA CORONACION, ANGELO ALESSANDRO</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>987 635 804</t>
+          <t>907 474 380</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2783,12 +2788,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
+          <t>ARIZAPANA CORONACION, ANGELO ALESSANDRO</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>987 635 804</t>
+          <t>907 474 380</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2870,7 +2875,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -3104,12 +3114,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -4432,12 +4442,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -4693,12 +4698,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -4780,12 +4785,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -4867,12 +4872,12 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -5215,12 +5220,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -5465,12 +5470,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -5639,12 +5639,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -6074,12 +6074,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -6596,12 +6596,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -6770,12 +6770,12 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -7107,12 +7107,12 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
+          <t>ARIZAPANA CORONACION, ANGELO ALESSANDRO</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>987 635 804</t>
+          <t>907 474 380</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -7194,12 +7194,12 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -7281,12 +7281,12 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -7368,12 +7368,12 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -7455,12 +7455,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H83" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -7542,12 +7537,12 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -8042,12 +8037,12 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -8216,12 +8211,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H92" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -8901,12 +8891,12 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
+          <t>ARIZAPANA CORONACION, ANGELO ALESSANDRO</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>987 635 804</t>
+          <t>907 474 380</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -9488,12 +9478,12 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
+          <t>ARIZAPANA CORONACION, ANGELO ALESSANDRO</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>987 635 804</t>
+          <t>907 474 380</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -9749,12 +9739,12 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -9836,12 +9826,12 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -10184,7 +10174,12 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -12071,12 +12066,12 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
+          <t>ARIZAPANA CORONACION, ANGELO ALESSANDRO</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>987 635 804</t>
+          <t>907 474 380</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -13017,12 +13012,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H148" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -13104,12 +13094,7 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H149" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -13767,12 +13752,12 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -14688,12 +14673,12 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -14775,12 +14760,12 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -16384,7 +16369,12 @@
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
@@ -16598,12 +16588,7 @@
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H192" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -17011,12 +16996,7 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H197" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -17837,12 +17817,12 @@
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>SULCA NUÑEZ, DAVID ALEJANDRO</t>
+          <t>NAVARRO ORGONE, ALFREDO</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>994 101 509</t>
+          <t>991892546</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
@@ -18663,12 +18643,7 @@
       </c>
       <c r="G217" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H217" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I217" t="inlineStr">
@@ -19261,12 +19236,12 @@
       </c>
       <c r="G224" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H224" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I224" t="inlineStr">
@@ -19435,7 +19410,12 @@
       </c>
       <c r="G226" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I226" t="inlineStr">
@@ -19604,7 +19584,12 @@
       </c>
       <c r="G228" t="inlineStr">
         <is>
-          <t>CHUMPITAZ VARGAS, GEORGE BENSON</t>
+          <t>CHIPANA QUISPE, CHRISTIAN ALONSO</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>953 450 482</t>
         </is>
       </c>
       <c r="I228" t="inlineStr">
@@ -19675,7 +19660,12 @@
       </c>
       <c r="G229" t="inlineStr">
         <is>
-          <t>CHUMPITAZ VARGAS, GEORGE BENSON</t>
+          <t>CHIPANA QUISPE, CHRISTIAN ALONSO</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>953 450 482</t>
         </is>
       </c>
       <c r="I229" t="inlineStr">
@@ -23706,12 +23696,12 @@
       </c>
       <c r="G281" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H281" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I281" t="inlineStr">
@@ -24304,12 +24294,12 @@
       </c>
       <c r="G288" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I288" t="inlineStr">
@@ -24728,12 +24718,12 @@
       </c>
       <c r="G293" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I293" t="inlineStr">
@@ -25044,12 +25034,12 @@
       </c>
       <c r="G297" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I297" t="inlineStr">
@@ -25729,12 +25719,12 @@
       </c>
       <c r="G305" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I305" t="inlineStr">
@@ -25816,12 +25806,12 @@
       </c>
       <c r="G306" t="inlineStr">
         <is>
-          <t>SULCA NUÑEZ, DAVID ALEJANDRO</t>
+          <t>NAVARRO ORGONE, ALFREDO</t>
         </is>
       </c>
       <c r="H306" t="inlineStr">
         <is>
-          <t>994 101 509</t>
+          <t>991892546</t>
         </is>
       </c>
       <c r="I306" t="inlineStr">
@@ -26127,12 +26117,12 @@
       </c>
       <c r="G310" t="inlineStr">
         <is>
-          <t>SULCA NUÑEZ, DAVID ALEJANDRO</t>
+          <t>NAVARRO ORGONE, ALFREDO</t>
         </is>
       </c>
       <c r="H310" t="inlineStr">
         <is>
-          <t>994 101 509</t>
+          <t>991892546</t>
         </is>
       </c>
       <c r="I310" t="inlineStr">
@@ -26203,7 +26193,12 @@
       </c>
       <c r="G311" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I311" t="inlineStr">
@@ -26285,7 +26280,12 @@
       </c>
       <c r="G312" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I312" t="inlineStr">
@@ -26530,12 +26530,12 @@
       </c>
       <c r="G315" t="inlineStr">
         <is>
-          <t>SULCA NUÑEZ, DAVID ALEJANDRO</t>
+          <t>NAVARRO ORGONE, ALFREDO</t>
         </is>
       </c>
       <c r="H315" t="inlineStr">
         <is>
-          <t>994 101 509</t>
+          <t>991892546</t>
         </is>
       </c>
       <c r="I315" t="inlineStr">
@@ -27117,7 +27117,12 @@
       </c>
       <c r="G322" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I322" t="inlineStr">
@@ -27286,7 +27291,12 @@
       </c>
       <c r="G324" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I324" t="inlineStr">
@@ -27787,7 +27797,12 @@
       </c>
       <c r="G330" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H330" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I330" t="inlineStr">
@@ -27956,12 +27971,12 @@
       </c>
       <c r="G332" t="inlineStr">
         <is>
-          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
+          <t>ARIZAPANA CORONACION, ANGELO ALESSANDRO</t>
         </is>
       </c>
       <c r="H332" t="inlineStr">
         <is>
-          <t>987 635 804</t>
+          <t>907 474 380</t>
         </is>
       </c>
       <c r="I332" t="inlineStr">
@@ -29576,12 +29591,12 @@
       </c>
       <c r="G351" t="inlineStr">
         <is>
-          <t>SULCA NUÑEZ, DAVID ALEJANDRO</t>
+          <t>NAVARRO ORGONE, ALFREDO</t>
         </is>
       </c>
       <c r="H351" t="inlineStr">
         <is>
-          <t>994 101 509</t>
+          <t>991892546</t>
         </is>
       </c>
       <c r="I351" t="inlineStr">
@@ -29739,12 +29754,12 @@
       </c>
       <c r="G353" t="inlineStr">
         <is>
-          <t>SULCA NUÑEZ, DAVID ALEJANDRO</t>
+          <t>NAVARRO ORGONE, ALFREDO</t>
         </is>
       </c>
       <c r="H353" t="inlineStr">
         <is>
-          <t>994 101 509</t>
+          <t>991892546</t>
         </is>
       </c>
       <c r="I353" t="inlineStr">
@@ -30065,12 +30080,12 @@
       </c>
       <c r="G357" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H357" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I357" t="inlineStr">
@@ -31143,7 +31158,12 @@
       </c>
       <c r="G370" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H370" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I370" t="inlineStr">
@@ -31225,7 +31245,12 @@
       </c>
       <c r="G371" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H371" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I371" t="inlineStr">
@@ -31557,12 +31582,12 @@
       </c>
       <c r="G375" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H375" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I375" t="inlineStr">
@@ -35374,7 +35399,12 @@
       </c>
       <c r="G424" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H424" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I424" t="inlineStr">
@@ -36473,12 +36503,12 @@
       </c>
       <c r="G437" t="inlineStr">
         <is>
-          <t>SULCA NUÑEZ, DAVID ALEJANDRO</t>
+          <t>NAVARRO ORGONE, ALFREDO</t>
         </is>
       </c>
       <c r="H437" t="inlineStr">
         <is>
-          <t>994 101 509</t>
+          <t>991892546</t>
         </is>
       </c>
       <c r="I437" t="inlineStr">
@@ -37653,12 +37683,12 @@
       </c>
       <c r="G451" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H451" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I451" t="inlineStr">
@@ -38088,12 +38118,12 @@
       </c>
       <c r="G456" t="inlineStr">
         <is>
-          <t>SULCA NUÑEZ, DAVID ALEJANDRO</t>
+          <t>NAVARRO ORGONE, ALFREDO</t>
         </is>
       </c>
       <c r="H456" t="inlineStr">
         <is>
-          <t>994 101 509</t>
+          <t>991892546</t>
         </is>
       </c>
       <c r="I456" t="inlineStr">
@@ -38235,12 +38265,7 @@
       </c>
       <c r="G458" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H458" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I458" t="inlineStr">
@@ -38322,12 +38347,12 @@
       </c>
       <c r="G459" t="inlineStr">
         <is>
-          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
+          <t>ARIZAPANA CORONACION, ANGELO ALESSANDRO</t>
         </is>
       </c>
       <c r="H459" t="inlineStr">
         <is>
-          <t>987 635 804</t>
+          <t>907 474 380</t>
         </is>
       </c>
       <c r="I459" t="inlineStr">
@@ -38746,12 +38771,7 @@
       </c>
       <c r="G464" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H464" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I464" t="inlineStr">
@@ -39181,12 +39201,12 @@
       </c>
       <c r="G469" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H469" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I469" t="inlineStr">
@@ -39355,12 +39375,7 @@
       </c>
       <c r="G471" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H471" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I471" t="inlineStr">
@@ -39616,12 +39631,12 @@
       </c>
       <c r="G474" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H474" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I474" t="inlineStr">
@@ -39703,7 +39718,12 @@
       </c>
       <c r="G475" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H475" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I475" t="inlineStr">
@@ -39785,12 +39805,12 @@
       </c>
       <c r="G476" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H476" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I476" t="inlineStr">
@@ -41001,12 +41021,12 @@
       </c>
       <c r="G491" t="inlineStr">
         <is>
-          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
+          <t>ARIZAPANA CORONACION, ANGELO ALESSANDRO</t>
         </is>
       </c>
       <c r="H491" t="inlineStr">
         <is>
-          <t>987 635 804</t>
+          <t>907 474 380</t>
         </is>
       </c>
       <c r="I491" t="inlineStr">
@@ -41262,12 +41282,7 @@
       </c>
       <c r="G494" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H494" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I494" t="inlineStr">
@@ -43002,7 +43017,12 @@
       </c>
       <c r="G514" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H514" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I514" t="inlineStr">
@@ -43606,12 +43626,12 @@
       </c>
       <c r="G521" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H521" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I521" t="inlineStr">
@@ -43943,12 +43963,12 @@
       </c>
       <c r="G525" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H525" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I525" t="inlineStr">
@@ -44204,12 +44224,12 @@
       </c>
       <c r="G528" t="inlineStr">
         <is>
-          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
+          <t>ARIZAPANA CORONACION, ANGELO ALESSANDRO</t>
         </is>
       </c>
       <c r="H528" t="inlineStr">
         <is>
-          <t>987 635 804</t>
+          <t>907 474 380</t>
         </is>
       </c>
       <c r="I528" t="inlineStr">
@@ -44291,12 +44311,7 @@
       </c>
       <c r="G529" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H529" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I529" t="inlineStr">
@@ -45074,12 +45089,7 @@
       </c>
       <c r="G538" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H538" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I538" t="inlineStr">
@@ -45161,12 +45171,12 @@
       </c>
       <c r="G539" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H539" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I539" t="inlineStr">
@@ -45248,12 +45258,7 @@
       </c>
       <c r="G540" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H540" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I540" t="inlineStr">
@@ -45498,12 +45503,12 @@
       </c>
       <c r="G543" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H543" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I543" t="inlineStr">
@@ -45585,12 +45590,7 @@
       </c>
       <c r="G544" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H544" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I544" t="inlineStr">
@@ -45835,12 +45835,7 @@
       </c>
       <c r="G547" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H547" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I547" t="inlineStr">
@@ -46618,7 +46613,12 @@
       </c>
       <c r="G556" t="inlineStr">
         <is>
-          <t>CHUMPITAZ VARGAS, GEORGE BENSON</t>
+          <t>CHIPANA QUISPE, CHRISTIAN ALONSO</t>
+        </is>
+      </c>
+      <c r="H556" t="inlineStr">
+        <is>
+          <t>953 450 482</t>
         </is>
       </c>
       <c r="I556" t="inlineStr">
@@ -46950,12 +46950,12 @@
       </c>
       <c r="G560" t="inlineStr">
         <is>
-          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
+          <t>ARIZAPANA CORONACION, ANGELO ALESSANDRO</t>
         </is>
       </c>
       <c r="H560" t="inlineStr">
         <is>
-          <t>987 635 804</t>
+          <t>907 474 380</t>
         </is>
       </c>
       <c r="I560" t="inlineStr">
@@ -47548,12 +47548,12 @@
       </c>
       <c r="G567" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H567" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I567" t="inlineStr">
@@ -47635,7 +47635,12 @@
       </c>
       <c r="G568" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H568" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I568" t="inlineStr">
@@ -48152,12 +48157,12 @@
       </c>
       <c r="G574" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H574" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I574" t="inlineStr">
@@ -48750,12 +48755,12 @@
       </c>
       <c r="G581" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H581" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I581" t="inlineStr">
@@ -49598,12 +49603,7 @@
       </c>
       <c r="G591" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H591" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I591" t="inlineStr">
@@ -50109,12 +50109,12 @@
       </c>
       <c r="G597" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H597" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I597" t="inlineStr">
@@ -51207,12 +51207,12 @@
       </c>
       <c r="G610" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H610" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I610" t="inlineStr">
@@ -51381,12 +51381,12 @@
       </c>
       <c r="G612" t="inlineStr">
         <is>
-          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
+          <t>ARIZAPANA CORONACION, ANGELO ALESSANDRO</t>
         </is>
       </c>
       <c r="H612" t="inlineStr">
         <is>
-          <t>987 635 804</t>
+          <t>907 474 380</t>
         </is>
       </c>
       <c r="I612" t="inlineStr">
@@ -51555,7 +51555,12 @@
       </c>
       <c r="G614" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H614" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I614" t="inlineStr">
@@ -51637,12 +51642,12 @@
       </c>
       <c r="G615" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H615" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I615" t="inlineStr">
@@ -51724,7 +51729,12 @@
       </c>
       <c r="G616" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H616" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I616" t="inlineStr">
@@ -52241,12 +52251,12 @@
       </c>
       <c r="G622" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H622" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I622" t="inlineStr">
@@ -54111,12 +54121,12 @@
       </c>
       <c r="G644" t="inlineStr">
         <is>
-          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
+          <t>ARIZAPANA CORONACION, ANGELO ALESSANDRO</t>
         </is>
       </c>
       <c r="H644" t="inlineStr">
         <is>
-          <t>987 635 804</t>
+          <t>907 474 380</t>
         </is>
       </c>
       <c r="I644" t="inlineStr">
@@ -56828,12 +56838,7 @@
       </c>
       <c r="G677" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H677" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I677" t="inlineStr">
@@ -56915,7 +56920,12 @@
       </c>
       <c r="G678" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H678" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I678" t="inlineStr">
@@ -57334,12 +57344,12 @@
       </c>
       <c r="G683" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H683" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I683" t="inlineStr">
@@ -58530,12 +58540,12 @@
       </c>
       <c r="G697" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H697" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I697" t="inlineStr">
@@ -58617,12 +58627,12 @@
       </c>
       <c r="G698" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H698" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I698" t="inlineStr">
@@ -59139,12 +59149,7 @@
       </c>
       <c r="G704" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H704" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I704" t="inlineStr">
@@ -59487,7 +59492,12 @@
       </c>
       <c r="G708" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H708" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I708" t="inlineStr">
@@ -59743,12 +59753,12 @@
       </c>
       <c r="G711" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H711" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I711" t="inlineStr">
@@ -60167,7 +60177,12 @@
       </c>
       <c r="G716" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H716" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I716" t="inlineStr">
@@ -60510,7 +60525,12 @@
       </c>
       <c r="G720" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H720" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I720" t="inlineStr">
@@ -60679,12 +60699,12 @@
       </c>
       <c r="G722" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H722" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I722" t="inlineStr">
@@ -61625,7 +61645,12 @@
       </c>
       <c r="G733" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H733" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I733" t="inlineStr">
@@ -61794,12 +61819,12 @@
       </c>
       <c r="G735" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H735" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I735" t="inlineStr">
@@ -62142,7 +62167,12 @@
       </c>
       <c r="G739" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H739" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I739" t="inlineStr">
@@ -62485,12 +62515,12 @@
       </c>
       <c r="G743" t="inlineStr">
         <is>
-          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
+          <t>ARIZAPANA CORONACION, ANGELO ALESSANDRO</t>
         </is>
       </c>
       <c r="H743" t="inlineStr">
         <is>
-          <t>987 635 804</t>
+          <t>907 474 380</t>
         </is>
       </c>
       <c r="I743" t="inlineStr">
@@ -62572,12 +62602,12 @@
       </c>
       <c r="G744" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H744" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I744" t="inlineStr">
@@ -63165,12 +63195,12 @@
       </c>
       <c r="G751" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H751" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I751" t="inlineStr">
@@ -64622,7 +64652,12 @@
       </c>
       <c r="G768" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H768" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I768" t="inlineStr">
@@ -65400,12 +65435,12 @@
       </c>
       <c r="G777" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H777" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I777" t="inlineStr">
@@ -65922,12 +65957,12 @@
       </c>
       <c r="G783" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H783" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I783" t="inlineStr">
@@ -66694,7 +66729,12 @@
       </c>
       <c r="G792" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H792" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I792" t="inlineStr">
@@ -67211,12 +67251,12 @@
       </c>
       <c r="G798" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H798" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I798" t="inlineStr">
@@ -67298,12 +67338,12 @@
       </c>
       <c r="G799" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H799" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I799" t="inlineStr">
@@ -68244,7 +68284,12 @@
       </c>
       <c r="G810" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H810" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I810" t="inlineStr">
@@ -68500,12 +68545,12 @@
       </c>
       <c r="G813" t="inlineStr">
         <is>
-          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
+          <t>ARIZAPANA CORONACION, ANGELO ALESSANDRO</t>
         </is>
       </c>
       <c r="H813" t="inlineStr">
         <is>
-          <t>987 635 804</t>
+          <t>907 474 380</t>
         </is>
       </c>
       <c r="I813" t="inlineStr">
@@ -68674,12 +68719,7 @@
       </c>
       <c r="G815" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H815" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I815" t="inlineStr">
@@ -68761,7 +68801,12 @@
       </c>
       <c r="G816" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H816" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I816" t="inlineStr">
@@ -69626,12 +69671,7 @@
       </c>
       <c r="G826" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H826" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I826" t="inlineStr">
@@ -70496,12 +70536,12 @@
       </c>
       <c r="G836" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H836" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I836" t="inlineStr">
@@ -71268,12 +71308,7 @@
       </c>
       <c r="G845" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H845" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I845" t="inlineStr">
@@ -72127,12 +72162,12 @@
       </c>
       <c r="G855" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H855" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I855" t="inlineStr">
@@ -72562,12 +72597,7 @@
       </c>
       <c r="G860" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H860" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I860" t="inlineStr">
@@ -73062,12 +73092,12 @@
       </c>
       <c r="G866" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H866" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I866" t="inlineStr">
@@ -73660,12 +73690,12 @@
       </c>
       <c r="G873" t="inlineStr">
         <is>
-          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
+          <t>ARIZAPANA CORONACION, ANGELO ALESSANDRO</t>
         </is>
       </c>
       <c r="H873" t="inlineStr">
         <is>
-          <t>987 635 804</t>
+          <t>907 474 380</t>
         </is>
       </c>
       <c r="I873" t="inlineStr">
@@ -73747,12 +73777,12 @@
       </c>
       <c r="G874" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H874" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I874" t="inlineStr">
@@ -74356,12 +74386,12 @@
       </c>
       <c r="G881" t="inlineStr">
         <is>
-          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
+          <t>ARIZAPANA CORONACION, ANGELO ALESSANDRO</t>
         </is>
       </c>
       <c r="H881" t="inlineStr">
         <is>
-          <t>987 635 804</t>
+          <t>907 474 380</t>
         </is>
       </c>
       <c r="I881" t="inlineStr">
@@ -74617,12 +74647,7 @@
       </c>
       <c r="G884" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H884" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I884" t="inlineStr">
@@ -74791,7 +74816,12 @@
       </c>
       <c r="G886" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H886" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I886" t="inlineStr">
@@ -75047,12 +75077,12 @@
       </c>
       <c r="G889" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H889" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I889" t="inlineStr">
@@ -75569,12 +75599,12 @@
       </c>
       <c r="G895" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H895" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I895" t="inlineStr">
@@ -75917,12 +75947,7 @@
       </c>
       <c r="G899" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H899" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I899" t="inlineStr">
@@ -76439,12 +76464,7 @@
       </c>
       <c r="G905" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H905" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I905" t="inlineStr">
@@ -76526,12 +76546,12 @@
       </c>
       <c r="G906" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H906" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I906" t="inlineStr">
@@ -76787,12 +76807,12 @@
       </c>
       <c r="G909" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H909" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I909" t="inlineStr">
@@ -76961,7 +76981,12 @@
       </c>
       <c r="G911" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H911" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I911" t="inlineStr">
@@ -77478,12 +77503,12 @@
       </c>
       <c r="G917" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H917" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I917" t="inlineStr">
@@ -78239,12 +78264,12 @@
       </c>
       <c r="G926" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H926" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I926" t="inlineStr">
@@ -78587,12 +78612,7 @@
       </c>
       <c r="G930" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H930" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I930" t="inlineStr">
@@ -78674,12 +78694,7 @@
       </c>
       <c r="G931" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H931" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I931" t="inlineStr">
@@ -78761,12 +78776,7 @@
       </c>
       <c r="G932" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H932" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I932" t="inlineStr">
@@ -79022,7 +79032,12 @@
       </c>
       <c r="G935" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H935" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I935" t="inlineStr">
@@ -79278,12 +79293,12 @@
       </c>
       <c r="G938" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H938" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I938" t="inlineStr">
@@ -79865,12 +79880,12 @@
       </c>
       <c r="G945" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H945" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I945" t="inlineStr">
@@ -80898,7 +80913,12 @@
       </c>
       <c r="G957" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H957" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I957" t="inlineStr">
@@ -81056,12 +81076,12 @@
       </c>
       <c r="G959" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H959" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I959" t="inlineStr">
@@ -81475,12 +81495,12 @@
       </c>
       <c r="G964" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H964" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I964" t="inlineStr">
@@ -81736,12 +81756,12 @@
       </c>
       <c r="G967" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H967" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I967" t="inlineStr">
@@ -82073,12 +82093,7 @@
       </c>
       <c r="G971" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H971" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I971" t="inlineStr">
@@ -82334,12 +82349,7 @@
       </c>
       <c r="G974" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H974" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I974" t="inlineStr">
@@ -83280,7 +83290,12 @@
       </c>
       <c r="G985" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H985" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I985" t="inlineStr">
@@ -83449,12 +83464,12 @@
       </c>
       <c r="G987" t="inlineStr">
         <is>
-          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
+          <t>ARIZAPANA CORONACION, ANGELO ALESSANDRO</t>
         </is>
       </c>
       <c r="H987" t="inlineStr">
         <is>
-          <t>987 635 804</t>
+          <t>907 474 380</t>
         </is>
       </c>
       <c r="I987" t="inlineStr">
@@ -83873,12 +83888,7 @@
       </c>
       <c r="G992" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H992" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I992" t="inlineStr">
@@ -84297,12 +84307,12 @@
       </c>
       <c r="G997" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H997" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I997" t="inlineStr">
@@ -86091,12 +86101,7 @@
       </c>
       <c r="G1018" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H1018" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I1018" t="inlineStr">
@@ -86863,12 +86868,12 @@
       </c>
       <c r="G1027" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H1027" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I1027" t="inlineStr">
@@ -86950,12 +86955,12 @@
       </c>
       <c r="G1028" t="inlineStr">
         <is>
-          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
+          <t>ARIZAPANA CORONACION, ANGELO ALESSANDRO</t>
         </is>
       </c>
       <c r="H1028" t="inlineStr">
         <is>
-          <t>987 635 804</t>
+          <t>907 474 380</t>
         </is>
       </c>
       <c r="I1028" t="inlineStr">
@@ -87124,12 +87129,12 @@
       </c>
       <c r="G1030" t="inlineStr">
         <is>
-          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
+          <t>ARIZAPANA CORONACION, ANGELO ALESSANDRO</t>
         </is>
       </c>
       <c r="H1030" t="inlineStr">
         <is>
-          <t>987 635 804</t>
+          <t>907 474 380</t>
         </is>
       </c>
       <c r="I1030" t="inlineStr">
@@ -88581,7 +88586,12 @@
       </c>
       <c r="G1047" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H1047" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I1047" t="inlineStr">
@@ -89261,12 +89271,12 @@
       </c>
       <c r="G1055" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H1055" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I1055" t="inlineStr">
@@ -90120,12 +90130,7 @@
       </c>
       <c r="G1065" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H1065" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I1065" t="inlineStr">
@@ -90207,12 +90212,12 @@
       </c>
       <c r="G1066" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H1066" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I1066" t="inlineStr">
@@ -93360,12 +93365,12 @@
       </c>
       <c r="G1103" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H1103" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I1103" t="inlineStr">
@@ -93447,12 +93452,7 @@
       </c>
       <c r="G1104" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H1104" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I1104" t="inlineStr">
@@ -93784,12 +93784,7 @@
       </c>
       <c r="G1108" t="inlineStr">
         <is>
-          <t>CUEVA ORBEGOZO, ALFONSO ENRIQUE</t>
-        </is>
-      </c>
-      <c r="H1108" t="inlineStr">
-        <is>
-          <t>987 635 519</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I1108" t="inlineStr">
@@ -94480,12 +94475,12 @@
       </c>
       <c r="G1116" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H1116" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I1116" t="inlineStr">
@@ -94567,12 +94562,12 @@
       </c>
       <c r="G1117" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H1117" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I1117" t="inlineStr">
@@ -94654,12 +94649,12 @@
       </c>
       <c r="G1118" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H1118" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I1118" t="inlineStr">
@@ -94828,12 +94823,12 @@
       </c>
       <c r="G1120" t="inlineStr">
         <is>
-          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
+          <t>ARIZAPANA CORONACION, ANGELO ALESSANDRO</t>
         </is>
       </c>
       <c r="H1120" t="inlineStr">
         <is>
-          <t>987 635 804</t>
+          <t>907 474 380</t>
         </is>
       </c>
       <c r="I1120" t="inlineStr">
@@ -94915,12 +94910,12 @@
       </c>
       <c r="G1121" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H1121" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I1121" t="inlineStr">
@@ -95176,12 +95171,12 @@
       </c>
       <c r="G1124" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H1124" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I1124" t="inlineStr">
@@ -95263,12 +95258,12 @@
       </c>
       <c r="G1125" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H1125" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I1125" t="inlineStr">
@@ -95350,12 +95345,12 @@
       </c>
       <c r="G1126" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H1126" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I1126" t="inlineStr">
@@ -95524,7 +95519,12 @@
       </c>
       <c r="G1128" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H1128" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I1128" t="inlineStr">
@@ -97661,7 +97661,12 @@
       </c>
       <c r="G1153" t="inlineStr">
         <is>
-          <t>Franco Maravi</t>
+          <t>PONCE BENITO, MOISES WALTHER</t>
+        </is>
+      </c>
+      <c r="H1153" t="inlineStr">
+        <is>
+          <t>968 965 845</t>
         </is>
       </c>
       <c r="I1153" t="inlineStr">
@@ -97743,12 +97748,12 @@
       </c>
       <c r="G1154" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H1154" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I1154" t="inlineStr">
@@ -97917,12 +97922,12 @@
       </c>
       <c r="G1156" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H1156" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I1156" t="inlineStr">
@@ -98439,12 +98444,12 @@
       </c>
       <c r="G1162" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H1162" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I1162" t="inlineStr">
@@ -98700,12 +98705,12 @@
       </c>
       <c r="G1165" t="inlineStr">
         <is>
-          <t>CARI PEREZ, JUAN PABLO</t>
+          <t>MONTOYA CARRIZO JOSE DANIEL</t>
         </is>
       </c>
       <c r="H1165" t="inlineStr">
         <is>
-          <t>987 635 469</t>
+          <t>968 965 493</t>
         </is>
       </c>
       <c r="I1165" t="inlineStr">
@@ -98787,12 +98792,12 @@
       </c>
       <c r="G1166" t="inlineStr">
         <is>
-          <t>DELGADO VELASQUEZ JOHN ANTHONY</t>
+          <t>GUERRERO CUETO, JEFFERSON PAOLO</t>
         </is>
       </c>
       <c r="H1166" t="inlineStr">
         <is>
-          <t>987 636 091</t>
+          <t>987 635 804</t>
         </is>
       </c>
       <c r="I1166" t="inlineStr">

</xml_diff>